<commit_message>
2026 update week 2
</commit_message>
<xml_diff>
--- a/data-viz/schedule.xlsx
+++ b/data-viz/schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/airwin/git-repos/data-viz-course/data-viz/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED742CC-3759-B546-8E23-C7CF4CECE346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEE19E94-ABD1-9E41-9FE2-C62D0A4C248F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19500" xr2:uid="{D262D957-99A2-4240-BB5D-74EA57927089}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" xr2:uid="{D262D957-99A2-4240-BB5D-74EA57927089}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="215">
   <si>
     <t>Date</t>
   </si>
@@ -670,6 +670,15 @@
   </si>
   <si>
     <t>lessons/106b-using-LLM-to-learn.html</t>
+  </si>
+  <si>
+    <t>exercise</t>
+  </si>
+  <si>
+    <t>exercise_link</t>
+  </si>
+  <si>
+    <t>#task-1</t>
   </si>
 </sst>
 </file>
@@ -1046,7 +1055,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5054E2AF-B146-EF4C-9336-1C427A68EF7D}">
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
@@ -1054,10 +1063,10 @@
     <col min="3" max="3" width="11.6640625" style="1" customWidth="1"/>
     <col min="4" max="5" width="28.1640625" customWidth="1"/>
     <col min="6" max="6" width="7" customWidth="1"/>
-    <col min="10" max="10" width="19.83203125" customWidth="1"/>
+    <col min="12" max="12" width="19.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -1083,19 +1092,25 @@
         <v>133</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1115,16 +1130,18 @@
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
-      <c r="I2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J2" s="2" t="s">
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -1144,22 +1161,22 @@
       <c r="F3" s="2">
         <v>1</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="J3" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -1179,22 +1196,22 @@
       <c r="F4" s="2">
         <v>2</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>2</v>
       </c>
@@ -1214,24 +1231,24 @@
       <c r="F5" s="2">
         <v>3</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2" t="s">
+      <c r="L5" s="2"/>
+      <c r="M5" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -1251,22 +1268,22 @@
       <c r="F6" s="2">
         <v>4</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>2</v>
       </c>
@@ -1286,26 +1303,26 @@
       <c r="F7" s="2">
         <v>5</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="M7" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="N7" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>2</v>
       </c>
@@ -1331,8 +1348,10 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>3</v>
       </c>
@@ -1352,26 +1371,26 @@
       <c r="F9" s="2">
         <v>6</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J9" s="2" t="s">
+      <c r="K9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L9" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="M9" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="N9" s="2" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>3</v>
       </c>
@@ -1391,22 +1410,22 @@
       <c r="F10" s="2">
         <v>7</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J10" s="2" t="s">
+      <c r="K10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L10" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>3</v>
       </c>
@@ -1426,26 +1445,26 @@
       <c r="F11" s="2">
         <v>8</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L11" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="M11" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="N11" s="2" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>4</v>
       </c>
@@ -1471,8 +1490,10 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>4</v>
       </c>
@@ -1492,20 +1513,20 @@
       <c r="F13" s="2">
         <v>9</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="I13" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="J13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J13" s="2" t="s">
+      <c r="K13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L13" s="2" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>4</v>
       </c>
@@ -1519,14 +1540,14 @@
       <c r="D14" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="K14" s="2" t="s">
+      <c r="M14" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L14" s="2" t="s">
+      <c r="N14" s="2" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>4</v>
       </c>
@@ -1546,20 +1567,20 @@
       <c r="F15" s="2">
         <v>10</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="I15" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J15" s="2" t="s">
+      <c r="K15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L15" s="2" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>4</v>
       </c>
@@ -1579,12 +1600,12 @@
       <c r="F16" s="2">
         <v>11</v>
       </c>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>5</v>
       </c>
@@ -1604,22 +1625,22 @@
       <c r="F17" s="2">
         <v>12</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="I17" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I17" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J17" s="2" t="s">
+      <c r="K17" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L17" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>5</v>
       </c>
@@ -1639,22 +1660,22 @@
       <c r="F18" s="2">
         <v>13</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="I18" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="I18" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J18" s="2" t="s">
+      <c r="K18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L18" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>5</v>
       </c>
@@ -1674,26 +1695,26 @@
       <c r="F19" s="2">
         <v>14</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="I19" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="M19" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="N19" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>5</v>
       </c>
@@ -1713,22 +1734,22 @@
       <c r="F20" s="2">
         <v>15</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="I20" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="I20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J20" s="2" t="s">
+      <c r="K20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L20" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>5</v>
       </c>
@@ -1754,8 +1775,10 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>5</v>
       </c>
@@ -1781,8 +1804,10 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>6</v>
       </c>
@@ -1802,26 +1827,26 @@
       <c r="F23" s="2">
         <v>16</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="I23" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="J23" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I23" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J23" s="2" t="s">
+      <c r="K23" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L23" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="K23" s="2" t="s">
+      <c r="M23" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L23" s="2" t="s">
+      <c r="N23" s="2" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>6</v>
       </c>
@@ -1841,22 +1866,22 @@
       <c r="F24" s="2">
         <v>17</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="I24" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="J24" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I24" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J24" s="2" t="s">
+      <c r="K24" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L24" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>6</v>
       </c>
@@ -1876,22 +1901,22 @@
       <c r="F25" s="2">
         <v>18</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="I25" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="H25" s="2" t="s">
+      <c r="J25" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="I25" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J25" s="2" t="s">
+      <c r="K25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L25" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>7</v>
       </c>
@@ -1913,8 +1938,10 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>8</v>
       </c>
@@ -1940,8 +1967,10 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>8</v>
       </c>
@@ -1961,22 +1990,22 @@
       <c r="F28" s="2">
         <v>19</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="I28" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="J28" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="I28" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J28" s="2" t="s">
+      <c r="K28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L28" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>8</v>
       </c>
@@ -1996,22 +2025,22 @@
       <c r="F29" s="2">
         <v>20</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="I29" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="J29" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="I29" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J29" s="2" t="s">
+      <c r="K29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L29" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M29" s="2"/>
+      <c r="N29" s="2"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>8</v>
       </c>
@@ -2031,26 +2060,26 @@
       <c r="F30" s="2">
         <v>21</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="I30" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="J30" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="I30" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J30" s="2" t="s">
+      <c r="K30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L30" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="K30" s="2" t="s">
+      <c r="M30" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L30" s="2" t="s">
+      <c r="N30" s="2" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
         <v>8</v>
       </c>
@@ -2072,8 +2101,10 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>9</v>
       </c>
@@ -2095,12 +2126,14 @@
       <c r="H32" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M32" s="2"/>
+      <c r="N32" s="2"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
         <v>9</v>
       </c>
@@ -2118,12 +2151,14 @@
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="4"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>10</v>
       </c>
@@ -2145,20 +2180,22 @@
       </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
-      <c r="I34" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J34" s="2" t="s">
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L34" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="K34" s="2" t="s">
+      <c r="M34" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L34" s="2" t="s">
+      <c r="N34" s="2" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>10</v>
       </c>
@@ -2178,22 +2215,22 @@
       <c r="F35" s="2">
         <v>23</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="I35" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="J35" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I35" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J35" s="2" t="s">
+      <c r="K35" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L35" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
         <v>10</v>
       </c>
@@ -2213,22 +2250,22 @@
       <c r="F36" s="2">
         <v>24</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="I36" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="J36" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="I36" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J36" s="2" t="s">
+      <c r="K36" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L36" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
         <v>11</v>
       </c>
@@ -2248,26 +2285,26 @@
       <c r="F37" s="2">
         <v>25</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="I37" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="J37" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="I37" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J37" s="2" t="s">
+      <c r="K37" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L37" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="K37" s="2" t="s">
+      <c r="M37" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L37" s="2" t="s">
+      <c r="N37" s="2" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
         <v>11</v>
       </c>
@@ -2289,16 +2326,18 @@
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
-      <c r="I38" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J38" s="2" t="s">
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L38" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M38" s="2"/>
+      <c r="N38" s="2"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
         <v>11</v>
       </c>
@@ -2320,16 +2359,18 @@
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
-      <c r="I39" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J39" s="2" t="s">
+      <c r="I39" s="2"/>
+      <c r="J39" s="2"/>
+      <c r="K39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L39" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="K39" s="2"/>
-      <c r="L39" s="2"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M39" s="2"/>
+      <c r="N39" s="2"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
         <v>11</v>
       </c>
@@ -2355,8 +2396,10 @@
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M40" s="2"/>
+      <c r="N40" s="2"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>12</v>
       </c>
@@ -2376,26 +2419,26 @@
       <c r="F41" s="2">
         <v>28</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="I41" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H41" s="2" t="s">
+      <c r="J41" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I41" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J41" s="2" t="s">
+      <c r="K41" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L41" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="K41" s="2" t="s">
+      <c r="M41" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L41" s="2" t="s">
+      <c r="N41" s="2" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
         <v>12</v>
       </c>
@@ -2415,26 +2458,26 @@
       <c r="F42" s="2">
         <v>29</v>
       </c>
-      <c r="G42" s="2" t="s">
+      <c r="I42" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="H42" s="2" t="s">
+      <c r="J42" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="I42" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J42" s="2" t="s">
+      <c r="K42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L42" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="K42" s="2" t="s">
+      <c r="M42" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L42" s="2" t="s">
+      <c r="N42" s="2" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
         <v>12</v>
       </c>
@@ -2454,22 +2497,22 @@
       <c r="F43" s="2">
         <v>30</v>
       </c>
-      <c r="G43" s="2" t="s">
+      <c r="I43" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="H43" s="2" t="s">
+      <c r="J43" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="I43" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J43" s="2" t="s">
+      <c r="K43" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L43" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="K43" s="2"/>
-      <c r="L43" s="2"/>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M43" s="2"/>
+      <c r="N43" s="2"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
         <v>14</v>
       </c>
@@ -2495,8 +2538,10 @@
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M44" s="2"/>
+      <c r="N44" s="2"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
         <v>13</v>
       </c>
@@ -2516,26 +2561,26 @@
       <c r="F45" s="2">
         <v>31</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="I45" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H45" s="2" t="s">
+      <c r="J45" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I45" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J45" s="2" t="s">
+      <c r="K45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L45" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="K45" s="2" t="s">
+      <c r="M45" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L45" s="2" t="s">
+      <c r="N45" s="2" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
         <v>13</v>
       </c>
@@ -2555,26 +2600,26 @@
       <c r="F46" s="2">
         <v>32</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="I46" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="J46" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="I46" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J46" s="2" t="s">
+      <c r="K46" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L46" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="K46" s="2" t="s">
+      <c r="M46" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L46" s="2" t="s">
+      <c r="N46" s="2" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
         <v>13</v>
       </c>
@@ -2594,26 +2639,26 @@
       <c r="F47" s="2">
         <v>33</v>
       </c>
-      <c r="G47" s="2" t="s">
+      <c r="I47" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H47" s="2" t="s">
+      <c r="J47" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="I47" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J47" s="2" t="s">
+      <c r="K47" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L47" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="K47" s="2" t="s">
+      <c r="M47" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L47" s="2" t="s">
+      <c r="N47" s="2" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>14</v>
       </c>
@@ -2635,16 +2680,18 @@
       </c>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
-      <c r="I48" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J48" s="2" t="s">
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L48" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="K48" s="2"/>
-      <c r="L48" s="2"/>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M48" s="2"/>
+      <c r="N48" s="2"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>14</v>
       </c>
@@ -2666,20 +2713,22 @@
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
-      <c r="I49" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J49" s="2" t="s">
+      <c r="I49" s="2"/>
+      <c r="J49" s="2"/>
+      <c r="K49" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L49" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="K49" s="2" t="s">
+      <c r="M49" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L49" s="2" t="s">
+      <c r="N49" s="2" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>14</v>
       </c>
@@ -2701,16 +2750,18 @@
       </c>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
-      <c r="I50" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J50" s="2" t="s">
+      <c r="I50" s="2"/>
+      <c r="J50" s="2"/>
+      <c r="K50" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L50" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="K50" s="2"/>
-      <c r="L50" s="2"/>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M50" s="2"/>
+      <c r="N50" s="2"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>14</v>
       </c>
@@ -2724,15 +2775,15 @@
       <c r="D51" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="I51" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J51" s="2" t="s">
+      <c r="K51" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L51" s="2" t="s">
         <v>202</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L51">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N51">
     <sortCondition ref="A2:A51"/>
     <sortCondition ref="B2:B51"/>
   </sortState>

</xml_diff>